<commit_message>
Stand nach dem ersten Zusammensitzen
</commit_message>
<xml_diff>
--- a/Doku/Testplan.xlsx
+++ b/Doku/Testplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonasmuhlbach/Programs_VB/Spiel_1.0/Doku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92D7F824-CC12-8D43-A8C4-DCFB2F507FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57A586D-ED9A-DD4E-8A13-3877018A74A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16120" xr2:uid="{FE7696FD-3E9E-A242-81BB-4231A40AE5FF}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15980" xr2:uid="{FE7696FD-3E9E-A242-81BB-4231A40AE5FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Funktion</t>
   </si>
@@ -54,6 +54,36 @@
   </si>
   <si>
     <t>Kommentar</t>
+  </si>
+  <si>
+    <t>Bewegung des Spielers nach links durch klicken</t>
+  </si>
+  <si>
+    <t>Bewegung des Spielers nach rechts durch klicken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durch langes drücken bewegt sich der Spieler schneller </t>
+  </si>
+  <si>
+    <t>Bei berührung eines Hindernisses wird ein Leben abgezogen</t>
+  </si>
+  <si>
+    <t>Sobald die Leben auf  0 fallen kommt ein Game Over Bildschirm</t>
+  </si>
+  <si>
+    <t>Die Hindernissdichte geht nicht über 5 in einer Reihe</t>
+  </si>
+  <si>
+    <t>ein Hindernissblock ist maximal 9 Zeichen groß</t>
+  </si>
+  <si>
+    <t>Die Leben werden in der unteren Linke Ecke angezeigt</t>
+  </si>
+  <si>
+    <t>Die Geschwindigeit steigert sich im Laufe des Spiels</t>
+  </si>
+  <si>
+    <t>Die Dichte an Hindernissen steigern sich im Laufe des Games</t>
   </si>
 </sst>
 </file>
@@ -456,12 +486,12 @@
   <dimension ref="A1:I1048576"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="1" max="1" width="54.33203125" customWidth="1"/>
     <col min="2" max="2" width="2" style="2" customWidth="1"/>
     <col min="3" max="3" width="11.6640625" customWidth="1"/>
     <col min="4" max="4" width="12.5" customWidth="1"/>
     <col min="5" max="5" width="2.1640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="22.1640625" customWidth="1"/>
+    <col min="6" max="6" width="48.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -495,61 +525,81 @@
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
+      <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
+      <c r="A10" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
+      <c r="A11" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
+      <c r="A12" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="F12" s="4"/>

</xml_diff>